<commit_message>
Add new incident templates and analysis files for FY26 Q1
- Created new Excel file for phase 2 feedback analysis.
- Added multiple CSV files for incident templates covering various transaction references and corrections for FY26 Q1.
- Included corrections for seller and buyer identification codes with appropriate flags for agreement and suggested corrections.
</commit_message>
<xml_diff>
--- a/data/test/sample/replay/phase_2_feedback/1903a~G15~P2_30-39~35_3~KR Final Analysis_Data_1 OF 1.xlsx
+++ b/data/test/sample/replay/phase_2_feedback/1903a~G15~P2_30-39~35_3~KR Final Analysis_Data_1 OF 1.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CZ11"/>
+  <dimension ref="A1:CZ13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -660,7 +660,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>35_3|35_8</t>
+          <t>35_3</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -668,7 +668,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Net amount is more than 0.01% away from expected value.</t>
+          <t>Exact match Net=Consideration+Interest — no action.</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -691,11 +691,11 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Values Provided</t>
+          <t>Agree</t>
         </is>
       </c>
       <c r="L2" t="n">
-        <v>2001</v>
+        <v>1000</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -704,7 +704,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>SAMPLE_P2_35_3_001</t>
+          <t>TXN400</t>
         </is>
       </c>
       <c r="O2" t="b">
@@ -720,7 +720,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Equity — UK</t>
+          <t>Equity - UK</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -729,10 +729,10 @@
         </is>
       </c>
       <c r="T2" t="n">
-        <v>1234.56</v>
+        <v>1000</v>
       </c>
       <c r="U2" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="V2" t="inlineStr">
         <is>
@@ -741,7 +741,7 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>12.3456</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Net amount difference within tolerance — no action required.</t>
+          <t>Delta 0.005 within 0.01 tolerance — no action.</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -789,12 +789,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>No Change</t>
+          <t>Client review</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>2002</v>
+        <v>2000</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -812,7 +812,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>SAMPLE_P2_35_3_002</t>
+          <t>TXN401</t>
         </is>
       </c>
       <c r="O3" t="b">
@@ -828,19 +828,19 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Equity — US</t>
+          <t>Equity - UK</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>US4592001014</t>
+          <t>GB0007980591</t>
         </is>
       </c>
       <c r="T3" t="n">
-        <v>2500</v>
+        <v>1000</v>
       </c>
       <c r="U3" t="n">
-        <v>0.001</v>
+        <v>0.005</v>
       </c>
       <c r="V3" t="inlineStr">
         <is>
@@ -849,7 +849,7 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Net amount materially different from reported value.</t>
+          <t>Delta 0.01 at tolerance boundary — review.</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -897,7 +897,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3500.00</t>
+          <t>Client review</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -907,11 +907,11 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Disagree</t>
+          <t>Agree</t>
         </is>
       </c>
       <c r="L4" t="n">
-        <v>2003</v>
+        <v>3000</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -920,7 +920,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>SAMPLE_P2_35_3_003</t>
+          <t>TXN402</t>
         </is>
       </c>
       <c r="O4" t="b">
@@ -936,19 +936,19 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>Equity — EU</t>
+          <t>Equity - UK</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>DE0005140008</t>
+          <t>GB0007980591</t>
         </is>
       </c>
       <c r="T4" t="n">
-        <v>3499.85</v>
+        <v>1000</v>
       </c>
       <c r="U4" t="n">
-        <v>0.15</v>
+        <v>0.01</v>
       </c>
       <c r="V4" t="inlineStr">
         <is>
@@ -957,7 +957,7 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
@@ -967,12 +967,12 @@
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>17.4999</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>GBP</t>
         </is>
       </c>
     </row>
@@ -992,7 +992,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Net amount not reported.</t>
+          <t>Delta 0.02 exceeds 0.01 tolerance — correction required.</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -1013,8 +1013,13 @@
           <t>FALSE</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Values Provided</t>
+        </is>
+      </c>
       <c r="L5" t="n">
-        <v>2004</v>
+        <v>4000</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -1023,7 +1028,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>SAMPLE_P2_35_3_NOTFOUND</t>
+          <t>TXN403</t>
         </is>
       </c>
       <c r="O5" t="b">
@@ -1039,13 +1044,19 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>Equity — UK</t>
+          <t>Equity - UK</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>GB0031348658</t>
-        </is>
+          <t>GB0007980591</t>
+        </is>
+      </c>
+      <c r="T5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="U5" t="n">
+        <v>0.02</v>
       </c>
       <c r="V5" t="inlineStr">
         <is>
@@ -1054,7 +1065,7 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
@@ -1064,7 +1075,7 @@
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
@@ -1081,7 +1092,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>35_3|35_10</t>
+          <t>35_3</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1089,7 +1100,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Net amount slightly off — client partially agrees.</t>
+          <t>Negative interest — net amount matches — no action.</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1102,7 +1113,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>5000.00</t>
+          <t>Client review</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1112,11 +1123,11 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Partially Agree</t>
+          <t>Agree</t>
         </is>
       </c>
       <c r="L6" t="n">
-        <v>2005</v>
+        <v>5000</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -1125,7 +1136,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>SAMPLE_P2_35_3_005</t>
+          <t>TXN404</t>
         </is>
       </c>
       <c r="O6" t="b">
@@ -1141,19 +1152,19 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Equity — UK</t>
+          <t>Equity - UK</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>GB0005405286</t>
+          <t>GB0007980591</t>
         </is>
       </c>
       <c r="T6" t="n">
-        <v>4998.75</v>
+        <v>980</v>
       </c>
       <c r="U6" t="n">
-        <v>1.25</v>
+        <v>0</v>
       </c>
       <c r="V6" t="inlineStr">
         <is>
@@ -1162,7 +1173,7 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
-          <t>250</t>
+          <t>980</t>
         </is>
       </c>
       <c r="Y6" t="inlineStr">
@@ -1172,7 +1183,7 @@
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>9.8</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
@@ -1197,7 +1208,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Net amount corrected in previous phase.</t>
+          <t>Zero interest — net amount matches — no action.</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -1210,7 +1221,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>1000.00</t>
+          <t>Client review</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1224,7 +1235,7 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>2006</v>
+        <v>6000</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -1233,7 +1244,7 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>SAMPLE_P2_35_3_006</t>
+          <t>TXN405</t>
         </is>
       </c>
       <c r="O7" t="b">
@@ -1249,16 +1260,16 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>Equity — UK</t>
+          <t>Equity - UK</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>GB0002634946</t>
+          <t>GB0007980591</t>
         </is>
       </c>
       <c r="T7" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="U7" t="n">
         <v>0</v>
@@ -1270,7 +1281,7 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>500</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr">
@@ -1280,27 +1291,12 @@
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
           <t>GBP</t>
-        </is>
-      </c>
-      <c r="AB7" t="inlineStr">
-        <is>
-          <t>35_3</t>
-        </is>
-      </c>
-      <c r="AC7" t="inlineStr">
-        <is>
-          <t>Phase 1</t>
-        </is>
-      </c>
-      <c r="AD7" t="inlineStr">
-        <is>
-          <t>999.75</t>
         </is>
       </c>
     </row>
@@ -1320,7 +1316,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Net amount is negative — client to confirm.</t>
+          <t>All zero values — no action required.</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -1343,11 +1339,11 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Values Provided</t>
+          <t>Agree</t>
         </is>
       </c>
       <c r="L8" t="n">
-        <v>2007</v>
+        <v>7000</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -1356,7 +1352,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>SAMPLE_P2_35_3_007</t>
+          <t>TXN406</t>
         </is>
       </c>
       <c r="O8" t="b">
@@ -1372,19 +1368,19 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>Equity — UK</t>
+          <t>Equity - UK</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>GB0004544929</t>
+          <t>GB0007980591</t>
         </is>
       </c>
       <c r="T8" t="n">
-        <v>-875.5</v>
+        <v>0</v>
       </c>
       <c r="U8" t="n">
-        <v>0.03</v>
+        <v>0</v>
       </c>
       <c r="V8" t="inlineStr">
         <is>
@@ -1393,7 +1389,7 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>0</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr">
@@ -1403,7 +1399,7 @@
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>-17.51</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr">
@@ -1428,7 +1424,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Net amount is zero — trade may not need reporting.</t>
+          <t>Large trade — delta within 0.01% of net — no action.</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -1441,7 +1437,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>Client review</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1455,7 +1451,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>2008</v>
+        <v>8000</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -1464,7 +1460,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>SAMPLE_P2_35_3_008</t>
+          <t>TXN407</t>
         </is>
       </c>
       <c r="O9" t="b">
@@ -1480,19 +1476,19 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>Equity — UK</t>
+          <t>Equity - UK</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>GB0005603229</t>
+          <t>GB0007980591</t>
         </is>
       </c>
       <c r="T9" t="n">
-        <v>0</v>
+        <v>1000000</v>
       </c>
       <c r="U9" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="V9" t="inlineStr">
         <is>
@@ -1501,7 +1497,7 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1000000</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr">
@@ -1511,7 +1507,7 @@
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>10000.0</t>
         </is>
       </c>
       <c r="AA9" t="inlineStr">
@@ -1536,7 +1532,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Net amount is more than 0.01% off.</t>
+          <t>Large trade — delta 0.003 within tolerance — no action.</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -1549,7 +1545,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>750.00</t>
+          <t>Client review</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1559,11 +1555,11 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>Agree</t>
         </is>
       </c>
       <c r="L10" t="n">
-        <v>2009</v>
+        <v>9000</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -1572,7 +1568,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>SAMPLE_P2_35_3_009</t>
+          <t>TXN408</t>
         </is>
       </c>
       <c r="O10" t="b">
@@ -1588,19 +1584,19 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>Equity — US</t>
+          <t>Equity - UK</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>US0231351067</t>
+          <t>GB0007980591</t>
         </is>
       </c>
       <c r="T10" t="n">
-        <v>748.25</v>
+        <v>1000000</v>
       </c>
       <c r="U10" t="n">
-        <v>1.75</v>
+        <v>0.003</v>
       </c>
       <c r="V10" t="inlineStr">
         <is>
@@ -1609,7 +1605,7 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>1000000</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr">
@@ -1619,12 +1615,12 @@
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>4.9883</t>
+          <t>10000.0</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>GBP</t>
         </is>
       </c>
     </row>
@@ -1644,7 +1640,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Net amount delta exceeds reporting threshold.</t>
+          <t>Net amount could not be parsed — client to confirm.</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -1657,7 +1653,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>12000.00</t>
+          <t>Client review</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1666,7 +1662,7 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>2010</v>
+        <v>10000</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -1675,7 +1671,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>SAMPLE_P2_35_3_010</t>
+          <t>TXN409</t>
         </is>
       </c>
       <c r="O11" t="b">
@@ -1691,19 +1687,19 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Equity — UK</t>
+          <t>Equity - UK</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>GB0004082847</t>
+          <t>GB0007980591</t>
         </is>
       </c>
       <c r="T11" t="n">
-        <v>11985</v>
+        <v>0</v>
       </c>
       <c r="U11" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="V11" t="inlineStr">
         <is>
@@ -1712,7 +1708,7 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>0</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr">
@@ -1722,10 +1718,226 @@
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>23.97</t>
+          <t>0</t>
         </is>
       </c>
       <c r="AA11" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>35_3</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>35_3</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>11</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>High interest — net amount matches — no action.</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>11</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Net amount</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Client review</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Agree</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>11000</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>213800SAMPLE0001LEI1</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>TXN410</t>
+        </is>
+      </c>
+      <c r="O12" t="b">
+        <v>1</v>
+      </c>
+      <c r="P12" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Equity - UK</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>GB0007980591</t>
+        </is>
+      </c>
+      <c r="T12" t="n">
+        <v>2000</v>
+      </c>
+      <c r="U12" t="n">
+        <v>0</v>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>MntryValAmt</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>35_3</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>35_3</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>12</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Small amounts — net amount matches — no action.</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>12</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Net amount</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Client review</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Agree</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>12000</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>213800SAMPLE0001LEI1</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>TXN411</t>
+        </is>
+      </c>
+      <c r="O13" t="b">
+        <v>1</v>
+      </c>
+      <c r="P13" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Equity</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Equity - UK</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>GB0007980591</t>
+        </is>
+      </c>
+      <c r="T13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="U13" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>MntryValAmt</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>0.0003</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
         <is>
           <t>GBP</t>
         </is>

</xml_diff>